<commit_message>
Update GAM delta models
</commit_message>
<xml_diff>
--- a/results/model_results.xlsx
+++ b/results/model_results.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26924"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\howar\Documents\Oregon State\Snow_CrabSDM\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18793320-BDF4-4A1E-B7BE-AD7F587DABB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A46D2014-7BC7-4BBE-AD61-114E52A8AC4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GAM" sheetId="1" r:id="rId1"/>
@@ -210,43 +210,46 @@
     <t>64.9% (59.6%)</t>
   </si>
   <si>
-    <t>65.8% (61.9%)</t>
-  </si>
-  <si>
-    <t>42.1% (56.5%)</t>
-  </si>
-  <si>
     <t>* number in parentheses is presence-absence model</t>
   </si>
   <si>
-    <t>33.0% (51.3%)</t>
-  </si>
-  <si>
-    <t>47.9% (43.1%)</t>
-  </si>
-  <si>
-    <t>41.2% (55.9%)</t>
-  </si>
-  <si>
-    <t>61.2% (60.2%)</t>
-  </si>
-  <si>
-    <t>51.2% (47.1%)</t>
-  </si>
-  <si>
-    <t>48.9% (59.7%)</t>
-  </si>
-  <si>
     <t>BRT (full)</t>
   </si>
   <si>
     <t>BRT (forecast)</t>
+  </si>
+  <si>
+    <t>63.6% (60.9%)</t>
+  </si>
+  <si>
+    <t>65.8% (62.2%)</t>
+  </si>
+  <si>
+    <t>42.2% (56.3%)</t>
+  </si>
+  <si>
+    <t>52.0% (47.8%)</t>
+  </si>
+  <si>
+    <t>49.0% (54.2%)</t>
+  </si>
+  <si>
+    <t>32.5% (55.6%)</t>
+  </si>
+  <si>
+    <t>47.9% (46.6%)</t>
+  </si>
+  <si>
+    <t>41.0% (59.9%)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -308,7 +311,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -318,6 +321,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -468,13 +472,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>2.61</c:v>
+                  <c:v>2.68</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>2.73</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.73</c:v>
+                  <c:v>1.72</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>2.31</c:v>
@@ -539,13 +543,13 @@
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>1.79</c:v>
+                  <c:v>1.86</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.72</c:v>
+                  <c:v>1.66</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.26</c:v>
+                  <c:v>1.24</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>1.69</c:v>
@@ -610,16 +614,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>1.68</c:v>
+                  <c:v>1.69</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.41</c:v>
+                  <c:v>1.42</c:v>
                 </c:pt>
-                <c:pt idx="2">
-                  <c:v>1.25</c:v>
+                <c:pt idx="2" formatCode="0.00">
+                  <c:v>1.2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.6</c:v>
+                  <c:v>1.58</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -791,6 +795,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -798,7 +803,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1678,21 +1682,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L31"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="9.6328125" customWidth="1"/>
-    <col min="3" max="3" width="10.81640625" customWidth="1"/>
-    <col min="4" max="4" width="71.08984375" customWidth="1"/>
-    <col min="6" max="6" width="5.90625" customWidth="1"/>
-    <col min="7" max="7" width="6.08984375" customWidth="1"/>
-    <col min="8" max="8" width="6.6328125" customWidth="1"/>
+    <col min="2" max="2" width="9.5703125" customWidth="1"/>
+    <col min="3" max="3" width="10.85546875" customWidth="1"/>
+    <col min="4" max="4" width="71.140625" customWidth="1"/>
+    <col min="6" max="6" width="5.85546875" customWidth="1"/>
+    <col min="7" max="7" width="6.140625" customWidth="1"/>
+    <col min="8" max="8" width="6.5703125" customWidth="1"/>
     <col min="9" max="9" width="4" customWidth="1"/>
-    <col min="10" max="10" width="12.54296875" customWidth="1"/>
+    <col min="10" max="10" width="12.5703125" customWidth="1"/>
     <col min="11" max="11" width="4" customWidth="1"/>
-    <col min="12" max="12" width="5.6328125" customWidth="1"/>
+    <col min="12" max="12" width="5.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -1730,7 +1734,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>25</v>
       </c>
@@ -1768,7 +1772,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>25</v>
       </c>
@@ -1806,7 +1810,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>25</v>
       </c>
@@ -1844,7 +1848,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>25</v>
       </c>
@@ -1879,7 +1883,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>25</v>
       </c>
@@ -1914,7 +1918,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>25</v>
       </c>
@@ -1949,7 +1953,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>26</v>
       </c>
@@ -1987,7 +1991,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>26</v>
       </c>
@@ -2025,7 +2029,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>26</v>
       </c>
@@ -2063,7 +2067,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>26</v>
       </c>
@@ -2098,7 +2102,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>26</v>
       </c>
@@ -2130,7 +2134,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>26</v>
       </c>
@@ -2165,7 +2169,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
         <v>25</v>
       </c>
@@ -2191,7 +2195,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
         <v>25</v>
       </c>
@@ -2226,7 +2230,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>25</v>
       </c>
@@ -2264,7 +2268,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
         <v>25</v>
       </c>
@@ -2287,7 +2291,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>25</v>
       </c>
@@ -2319,7 +2323,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>25</v>
       </c>
@@ -2354,7 +2358,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>26</v>
       </c>
@@ -2380,7 +2384,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>26</v>
       </c>
@@ -2415,7 +2419,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>26</v>
       </c>
@@ -2453,7 +2457,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
         <v>26</v>
       </c>
@@ -2476,7 +2480,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>26</v>
       </c>
@@ -2508,7 +2512,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
         <v>26</v>
       </c>
@@ -2543,17 +2547,17 @@
         <v>21</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="K29" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="K30" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="K31" t="s">
         <v>14</v>
       </c>
@@ -2567,19 +2571,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C28747FF-1FB7-4EF0-9863-442B02C2FB9C}">
   <dimension ref="A1:I25"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="25.08984375" customWidth="1"/>
-    <col min="3" max="3" width="13.90625" customWidth="1"/>
-    <col min="4" max="4" width="12.6328125" customWidth="1"/>
-    <col min="5" max="5" width="11.7265625" customWidth="1"/>
-    <col min="6" max="6" width="15.54296875" customWidth="1"/>
-    <col min="7" max="7" width="10.90625" customWidth="1"/>
-    <col min="8" max="8" width="17.1796875" customWidth="1"/>
-    <col min="9" max="9" width="12.90625" customWidth="1"/>
+    <col min="2" max="2" width="25.140625" customWidth="1"/>
+    <col min="3" max="3" width="13.85546875" customWidth="1"/>
+    <col min="4" max="4" width="12.5703125" customWidth="1"/>
+    <col min="5" max="5" width="11.7109375" customWidth="1"/>
+    <col min="6" max="6" width="15.5703125" customWidth="1"/>
+    <col min="7" max="7" width="10.85546875" customWidth="1"/>
+    <col min="8" max="8" width="17.140625" customWidth="1"/>
+    <col min="9" max="9" width="12.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -2608,7 +2612,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>25</v>
       </c>
@@ -2637,7 +2641,7 @@
         <v>0.56000000000000005</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>25</v>
       </c>
@@ -2666,7 +2670,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>25</v>
       </c>
@@ -2695,7 +2699,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>25</v>
       </c>
@@ -2724,7 +2728,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>25</v>
       </c>
@@ -2753,7 +2757,7 @@
         <v>0.48</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>25</v>
       </c>
@@ -2782,7 +2786,7 @@
         <v>0.84</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>25</v>
       </c>
@@ -2811,7 +2815,7 @@
         <v>0.42</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>25</v>
       </c>
@@ -2819,82 +2823,82 @@
         <v>53</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
         <v>26</v>
       </c>
@@ -2908,19 +2912,19 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E502E113-8B3D-455D-A134-6030657C990C}">
   <dimension ref="B1:L17"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="17.1796875" customWidth="1"/>
-    <col min="3" max="3" width="13.6328125" customWidth="1"/>
-    <col min="4" max="4" width="12.54296875" customWidth="1"/>
+    <col min="2" max="2" width="17.140625" customWidth="1"/>
+    <col min="3" max="3" width="13.5703125" customWidth="1"/>
+    <col min="4" max="4" width="12.5703125" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="8" max="8" width="16.26953125" customWidth="1"/>
+    <col min="8" max="8" width="16.28515625" customWidth="1"/>
     <col min="9" max="9" width="14" customWidth="1"/>
-    <col min="10" max="10" width="13.7265625" customWidth="1"/>
-    <col min="11" max="11" width="13.1796875" customWidth="1"/>
+    <col min="10" max="10" width="13.7109375" customWidth="1"/>
+    <col min="11" max="11" width="13.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="C1" t="s">
         <v>41</v>
       </c>
@@ -2928,7 +2932,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
       <c r="C3" s="1" t="s">
         <v>38</v>
       </c>
@@ -2951,36 +2955,36 @@
         <v>55</v>
       </c>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>34</v>
       </c>
       <c r="C4">
-        <v>2.61</v>
+        <v>2.68</v>
       </c>
       <c r="D4" s="8">
-        <v>1.79</v>
+        <v>1.86</v>
       </c>
       <c r="E4">
-        <v>1.68</v>
+        <v>1.69</v>
       </c>
       <c r="H4" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="I4" s="2">
-        <v>0.61299999999999999</v>
+      <c r="I4" s="9">
+        <v>0.60799999999999998</v>
       </c>
       <c r="J4" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="K4" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="L4" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>35</v>
       </c>
@@ -2988,57 +2992,57 @@
         <v>2.73</v>
       </c>
       <c r="D5" s="8">
-        <v>1.72</v>
+        <v>1.66</v>
       </c>
       <c r="E5">
-        <v>1.41</v>
+        <v>1.42</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="I5" s="2">
-        <v>0.68700000000000006</v>
+      <c r="I5" s="9">
+        <v>0.68600000000000005</v>
       </c>
       <c r="J5" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="K5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="L5" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
         <v>36</v>
       </c>
       <c r="C6">
-        <v>1.73</v>
+        <v>1.72</v>
       </c>
       <c r="D6" s="8">
-        <v>1.26</v>
-      </c>
-      <c r="E6">
-        <v>1.25</v>
+        <v>1.24</v>
+      </c>
+      <c r="E6" s="8">
+        <v>1.2</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="I6" s="2">
-        <v>0.61599999999999999</v>
+      <c r="I6" s="9">
+        <v>0.61399999999999999</v>
       </c>
       <c r="J6" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="K6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="L6" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
         <v>37</v>
       </c>
@@ -3049,35 +3053,35 @@
         <v>1.69</v>
       </c>
       <c r="E7">
-        <v>1.6</v>
+        <v>1.58</v>
       </c>
       <c r="H7" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="I7" s="2">
-        <v>0.71199999999999997</v>
+      <c r="I7" s="9">
+        <v>0.70899999999999996</v>
       </c>
       <c r="J7" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="K7" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="L7" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
       <c r="J10" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
       <c r="I12" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
       <c r="I13" s="1" t="s">
         <v>38</v>
       </c>
@@ -3088,35 +3092,35 @@
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
       <c r="H14" s="1" t="s">
         <v>34</v>
       </c>
       <c r="I14" s="8">
-        <v>0.64</v>
+        <v>0.63</v>
       </c>
       <c r="J14" s="8">
-        <v>0.67</v>
+        <v>0.68</v>
       </c>
       <c r="K14" s="8">
         <v>0.69</v>
       </c>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
       <c r="H15" s="1" t="s">
         <v>35</v>
       </c>
       <c r="I15" s="8">
-        <v>0.48</v>
+        <v>0.66</v>
       </c>
       <c r="J15" s="8">
-        <v>0.55000000000000004</v>
+        <v>0.7</v>
       </c>
       <c r="K15" s="8">
-        <v>0.7</v>
-      </c>
-    </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
+        <v>0.71</v>
+      </c>
+    </row>
+    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
       <c r="H16" s="1" t="s">
         <v>36</v>
       </c>
@@ -3124,24 +3128,24 @@
         <v>0.75</v>
       </c>
       <c r="J16" s="8">
-        <v>0.75</v>
+        <v>0.76</v>
       </c>
       <c r="K16" s="8">
-        <v>0.76</v>
-      </c>
-    </row>
-    <row r="17" spans="8:11" x14ac:dyDescent="0.35">
+        <v>0.77</v>
+      </c>
+    </row>
+    <row r="17" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H17" s="1" t="s">
         <v>37</v>
       </c>
       <c r="I17" s="8">
-        <v>0.78</v>
+        <v>0.79</v>
       </c>
       <c r="J17" s="8">
-        <v>0.79</v>
+        <v>0.82</v>
       </c>
       <c r="K17" s="8">
-        <v>0.82</v>
+        <v>0.83</v>
       </c>
     </row>
   </sheetData>
@@ -3154,27 +3158,27 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8220CFE4-3936-4A88-B5F4-62055CA5BCB2}">
   <dimension ref="B1:D7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="16.453125" customWidth="1"/>
-    <col min="3" max="3" width="13.54296875" customWidth="1"/>
-    <col min="4" max="4" width="12.453125" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" customWidth="1"/>
+    <col min="3" max="3" width="13.5703125" customWidth="1"/>
+    <col min="4" max="4" width="12.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C3" s="1" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>34</v>
       </c>
@@ -3185,7 +3189,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>35</v>
       </c>
@@ -3196,7 +3200,7 @@
         <v>1.32</v>
       </c>
     </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
         <v>36</v>
       </c>
@@ -3207,7 +3211,7 @@
         <v>1.05</v>
       </c>
     </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
         <v>37</v>
       </c>

</xml_diff>